<commit_message>
more datacamp and disk_savvy data
</commit_message>
<xml_diff>
--- a/datacamp.xlsx
+++ b/datacamp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Desktop\NAUKA\Python Nauka\data_science\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24523501-88AC-4A73-93A0-A6F46F0CD139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62730695-695D-40EC-942A-59DACE7F7E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="5085" windowHeight="9375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3285" yWindow="3285" windowWidth="5085" windowHeight="9375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -343,12 +343,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="537" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="538" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4659,11 +4667,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="538">
+  <cellXfs count="539">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="534" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="533" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="535" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="532" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="534" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="531" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="530" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="529" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4679,10 +4688,10 @@
     <xf numFmtId="0" fontId="519" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="518" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="517" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="516" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="534" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="535" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="516" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="515" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="514" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="513" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4942,9 +4951,9 @@
     <xf numFmtId="0" fontId="259" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="258" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="257" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="536" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="537" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="256" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="535" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="536" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="255" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="254" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="253" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6116,6 +6125,9 @@
       <c r="W14" s="474">
         <v>4</v>
       </c>
+      <c r="X14" s="538">
+        <v>5</v>
+      </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">

</xml_diff>